<commit_message>
Populate IQIYI FY2024 + 2025 financials
</commit_message>
<xml_diff>
--- a/models/builds/2026-05-14-phuong-iqiyi-financials.xlsx
+++ b/models/builds/2026-05-14-phuong-iqiyi-financials.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luongduyphuong/Documents/GitHub/Corporate-Finance-/models/builds/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luongduyphuong/Library/CloudStorage/GoogleDrive-duyphuonglt@gmail.com/My Drive/Vemba/Bus 629 finance /Corporate-Finance-/models/builds/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4718372-EDA2-7149-B00B-F961C9580D7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2196377A-FA16-794E-B3CB-651CD4612747}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -66,8 +66,9 @@
     <definedName name="BAL_receivables_prior">'Balance Sheet'!$D$8</definedName>
     <definedName name="BAL_retained_earnings_curr">'Balance Sheet'!$G$19</definedName>
     <definedName name="BAL_retained_earnings_prior">'Balance Sheet'!$H$19</definedName>
-    <definedName name="CASH_investments">'Cash Flow Statement'!$C$22</definedName>
-    <definedName name="CASH_operating">'Cash Flow Statement'!$C$16</definedName>
+    <definedName name="CASH_investments">'Cash Flow Statement'!$C$23</definedName>
+    <definedName name="CASH_operating">'Cash Flow Statement'!$C$17</definedName>
+    <definedName name="CF_depreciation_amortization">'Cash Flow Statement'!$C$8</definedName>
     <definedName name="cost_capital">Ratios!$C$10</definedName>
     <definedName name="currentYear_after_tax_operating_income">Ratios!$C$22</definedName>
     <definedName name="currentYear_assets_current">Ratios!$C$26</definedName>
@@ -299,11 +300,20 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-Source: SEC EDGAR, accession 000119312526107079</t>
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Source: SEC EDGAR, accession 000119312526107079</t>
         </r>
       </text>
     </comment>
-    <comment ref="C10" authorId="0" shapeId="0" xr:uid="{BA50804D-676A-9D45-B6CA-13DB09C3CDCB}">
+    <comment ref="C11" authorId="0" shapeId="0" xr:uid="{BA50804D-676A-9D45-B6CA-13DB09C3CDCB}">
       <text>
         <r>
           <rPr>
@@ -336,7 +346,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C11" authorId="0" shapeId="0" xr:uid="{267B063F-1087-E547-ABB2-31DE89ABFFA9}">
+    <comment ref="C12" authorId="0" shapeId="0" xr:uid="{267B063F-1087-E547-ABB2-31DE89ABFFA9}">
       <text>
         <r>
           <rPr>
@@ -369,7 +379,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C12" authorId="0" shapeId="0" xr:uid="{F65496A6-BFF1-0146-B894-B380E1BC31D7}">
+    <comment ref="C13" authorId="0" shapeId="0" xr:uid="{F65496A6-BFF1-0146-B894-B380E1BC31D7}">
       <text>
         <r>
           <rPr>
@@ -402,7 +412,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C13" authorId="0" shapeId="0" xr:uid="{4120681A-6AAF-424F-8C90-F7A07490679B}">
+    <comment ref="C14" authorId="0" shapeId="0" xr:uid="{4120681A-6AAF-424F-8C90-F7A07490679B}">
       <text>
         <r>
           <rPr>
@@ -435,7 +445,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C14" authorId="0" shapeId="0" xr:uid="{83B74DC5-4749-7E41-BF5E-C6E6AB7DE60D}">
+    <comment ref="C15" authorId="0" shapeId="0" xr:uid="{83B74DC5-4749-7E41-BF5E-C6E6AB7DE60D}">
       <text>
         <r>
           <rPr>
@@ -473,7 +483,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="350">
   <si>
     <t>Ratios &amp; Derived Inputs</t>
   </si>
@@ -514,9 +524,6 @@
     <t>share_price</t>
   </si>
   <si>
-    <t>Shares outstanding (M)</t>
-  </si>
-  <si>
     <t>shares_outstanding</t>
   </si>
   <si>
@@ -883,9 +890,6 @@
     <t>Cash coverage ratio</t>
   </si>
   <si>
-    <t>(INC_ebit + INC_depreciation) / INC_interest_expense</t>
-  </si>
-  <si>
     <t>Debt burden</t>
   </si>
   <si>
@@ -1357,12 +1361,6 @@
     <t>Fiscal Year (prior)</t>
   </si>
   <si>
-    <t>Data Source</t>
-  </si>
-  <si>
-    <t>[SEC EDGAR 10-K URL / Yahoo Finance / etc.]</t>
-  </si>
-  <si>
     <t>Units</t>
   </si>
   <si>
@@ -1462,9 +1460,6 @@
     <t>FY2024 (fiscal year ended December 31, 2024)</t>
   </si>
   <si>
-    <t>SEC EDGAR — Form 20-F (FY2025), CIK 1722608. URL: https://www.sec.gov/Archives/edgar/data/1722608/000119312526107079/iq-20251231.htm</t>
-  </si>
-  <si>
     <t>All figures in RMB thousands (RMB '000) unless otherwise noted. USD figures translated at RMB6.9956 = US$1.00 (Dec 31, 2025 rate per 20-F).</t>
   </si>
   <si>
@@ -1484,6 +1479,63 @@
   </si>
   <si>
     <t>In progress</t>
+  </si>
+  <si>
+    <t>Done
+https://github.com/duyphuonglt-gif/Corporate-Finance-/blob/main/models/builds/2026-05-14-phuong-iqiyi-financials.xlsx</t>
+  </si>
+  <si>
+    <t>plus Other non-cash adjustments</t>
+  </si>
+  <si>
+    <t>[20-F: provision for credit losses, unrealized FX, accretion on notes, barter, SBC, equity method, impairments, deferred tax, other]</t>
+  </si>
+  <si>
+    <t>CF Depreciation correction</t>
+  </si>
+  <si>
+    <t>Cash Flow Statement row 8 corrected from 13,363,219 → 13,264,120 (pure D&amp;A only: fixed assets 138,337 + intangibles 75,634 + licensed copyrights 6,137,566 + produced content 6,912,583 = 13,264,120). Bundled non-cash items (99,099) moved to new row 9 'Other non-cash adjustments'. Net cash from operations unchanged at 105,801.</t>
+  </si>
+  <si>
+    <t>Source: SEC EDGAR Form 20-F FY2025, Consolidated Statements of Cash Flows (F-8 to F-9)</t>
+  </si>
+  <si>
+    <t>PP&amp;E reported net in 20-F Note 11; gross cost &amp; accumulated depreciation not disclosed separately in primary statements.</t>
+  </si>
+  <si>
+    <t>Net PP&amp;E = gross cost less accumulated depreciation (combined). See 20-F Note 11 for asset category breakdown.</t>
+  </si>
+  <si>
+    <t>Shares outstanding ('000 ADS)</t>
+  </si>
+  <si>
+    <t>1 ADS = 7 Class A ordinary shares. 6,754,381,564 total ordinary shares ÷ 7 = ~964,912K ADS. Ratios tab uses diluted wt-avg basis: 6,746,355,442 ord. shares ÷ 7 = 963,765K ADS ≈ 962,959K ADS entered. Share price US$1.18; market cap = 1.18 × 962,959 = US$1,136,292K (~US$1.1B).</t>
+  </si>
+  <si>
+    <t>(INC_ebit + CF_depreciation_amortization) / INC_interest_expense</t>
+  </si>
+  <si>
+    <t>CF_depreciation_amortization = total D&amp;A from CF Statement (13,264,120); D&amp;A not broken out on IS as iQIYI embeds it in cost lines</t>
+  </si>
+  <si>
+    <t>Data Source &amp; Filing Type</t>
+  </si>
+  <si>
+    <t>SEC EDGAR — Form 20-F (FY2025), CIK 1722608.
+URL: https://www.sec.gov/Archives/edgar/data/1722608/000119312526107079/iq-20251231.htm
+NOTE — Non-US Filing: Form 20-F is the SEC annual report for Foreign Private Issuers; it is the functional equivalent of a Form 10-K for non-US companies listed on US exchanges. iQIYI, Inc. is a Cayman Islands-incorporated company with principal operations in the PRC, listed on Nasdaq as a Foreign Private Issuer.</t>
+  </si>
+  <si>
+    <t>SEC EDGAR 20-F URL / accession 000119312526107079</t>
+  </si>
+  <si>
+    <t>Reporting Standard</t>
+  </si>
+  <si>
+    <t>US GAAP (United States Generally Accepted Accounting Principles), as required for SEC registrants filing on Form 20-F. Financial statements prepared in accordance with FASB ASC standards. iQIYI elected to use US GAAP rather than IFRS as permitted for Foreign Private Issuers.</t>
+  </si>
+  <si>
+    <t>Source: 20-F Cover Page — 'The financial statements are prepared in accordance with US GAAP'</t>
   </si>
 </sst>
 </file>
@@ -1500,7 +1552,7 @@
     <numFmt numFmtId="170" formatCode="0.0&quot; days&quot;"/>
     <numFmt numFmtId="171" formatCode="0.000"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1625,6 +1677,19 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Open Sans"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="8"/>
+      <color rgb="FF808080"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -1697,7 +1762,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1777,17 +1842,21 @@
     <xf numFmtId="49" fontId="18" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1803,10 +1872,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2130,22 +2195,22 @@
       <c r="C2" s="1"/>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B4" s="47" t="s">
-        <v>157</v>
-      </c>
-      <c r="C4" s="46"/>
+      <c r="B4" s="46" t="s">
+        <v>155</v>
+      </c>
+      <c r="C4" s="47"/>
     </row>
     <row r="5" spans="2:3" ht="26" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="50" t="s">
-        <v>158</v>
-      </c>
-      <c r="C5" s="46"/>
+        <v>156</v>
+      </c>
+      <c r="C5" s="47"/>
     </row>
     <row r="6" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="48" t="s">
-        <v>159</v>
-      </c>
-      <c r="C6" s="46"/>
+        <v>157</v>
+      </c>
+      <c r="C6" s="47"/>
     </row>
     <row r="7" spans="2:3" ht="4" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="2"/>
@@ -2153,209 +2218,209 @@
     </row>
     <row r="9" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="49" t="s">
-        <v>160</v>
-      </c>
-      <c r="C9" s="46"/>
+        <v>158</v>
+      </c>
+      <c r="C9" s="47"/>
     </row>
     <row r="10" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="14" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="15" spans="2:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="49" t="s">
-        <v>173</v>
-      </c>
-      <c r="C17" s="46"/>
+        <v>171</v>
+      </c>
+      <c r="C17" s="47"/>
     </row>
     <row r="18" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="19" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="6" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="8" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="9" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="22" spans="2:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="10" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="24" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="49" t="s">
-        <v>184</v>
-      </c>
-      <c r="C24" s="46"/>
+        <v>182</v>
+      </c>
+      <c r="C24" s="47"/>
     </row>
     <row r="25" spans="2:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="5" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="26" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="11" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="11" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="28" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="11" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="29" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="11" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="30" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="11" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="11" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="32" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="11" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="33" spans="2:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="11" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="36" spans="2:3" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B36" s="49" t="s">
-        <v>202</v>
-      </c>
-      <c r="C36" s="46"/>
+        <v>200</v>
+      </c>
+      <c r="C36" s="47"/>
     </row>
     <row r="37" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="12" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="38" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="12" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B41" s="51" t="s">
-        <v>207</v>
-      </c>
-      <c r="C41" s="46"/>
+        <v>205</v>
+      </c>
+      <c r="C41" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -2387,45 +2452,45 @@
   <sheetData>
     <row r="2" spans="2:8" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B3" s="15" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="16" t="s">
+        <v>208</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>209</v>
+      </c>
+      <c r="D5" s="17" t="s">
         <v>210</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="F5" s="16" t="s">
         <v>211</v>
       </c>
-      <c r="D5" s="17" t="s">
-        <v>212</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>213</v>
-      </c>
       <c r="G5" s="17" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="18" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="12" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C7" s="19">
         <v>4354275</v>
@@ -2434,7 +2499,7 @@
         <v>3529679</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="G7" s="19">
         <v>4690642</v>
@@ -2445,7 +2510,7 @@
     </row>
     <row r="8" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="12" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C8" s="19">
         <v>2522668</v>
@@ -2454,7 +2519,7 @@
         <v>2191178</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="G8" s="19">
         <v>6652432</v>
@@ -2465,7 +2530,7 @@
     </row>
     <row r="9" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="12" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="C9" s="19">
         <v>447507</v>
@@ -2474,7 +2539,7 @@
         <v>388718</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="G9" s="19">
         <v>10724233</v>
@@ -2485,7 +2550,7 @@
     </row>
     <row r="10" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="12" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C10" s="19">
         <v>2965845</v>
@@ -2494,7 +2559,7 @@
         <v>3417661</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="G10" s="21">
         <f>SUM(G7:G9)</f>
@@ -2507,7 +2572,7 @@
     </row>
     <row r="11" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="20" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C11" s="21">
         <f>SUM(C7:C10)</f>
@@ -2520,7 +2585,7 @@
     </row>
     <row r="12" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F12" s="12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G12" s="19">
         <v>10080824</v>
@@ -2531,10 +2596,10 @@
     </row>
     <row r="13" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="18" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="G13" s="19">
         <v>1224678</v>
@@ -2545,7 +2610,7 @@
     </row>
     <row r="14" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="12" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C14" s="19">
         <v>903427</v>
@@ -2556,7 +2621,7 @@
     </row>
     <row r="15" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="12" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C15" s="19">
         <v>0</v>
@@ -2564,8 +2629,11 @@
       <c r="D15" s="19">
         <v>0</v>
       </c>
+      <c r="E15" s="55" t="s">
+        <v>338</v>
+      </c>
       <c r="F15" s="20" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="G15" s="21">
         <f>G10+G12+G13</f>
@@ -2578,7 +2646,7 @@
     </row>
     <row r="16" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="20" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C16" s="21">
         <f>C14-C15</f>
@@ -2588,18 +2656,21 @@
         <f>D14-D15</f>
         <v>877982</v>
       </c>
+      <c r="E16" s="55" t="s">
+        <v>339</v>
+      </c>
     </row>
     <row r="17" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F17" s="18" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="18" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="G18" s="19">
         <v>56026664</v>
@@ -2610,7 +2681,7 @@
     </row>
     <row r="19" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="12" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C19" s="19">
         <v>3820823</v>
@@ -2619,7 +2690,7 @@
         <v>3820823</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="G19" s="19">
         <v>-42717738</v>
@@ -2630,7 +2701,7 @@
     </row>
     <row r="20" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="12" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C20" s="19">
         <v>31667190</v>
@@ -2639,7 +2710,7 @@
         <v>31534484</v>
       </c>
       <c r="F20" s="20" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="G20" s="21">
         <f>G18+G19</f>
@@ -2653,7 +2724,7 @@
     <row r="22" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="23" spans="2:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="5" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C23" s="22">
         <f>C11+C16+C19+C20</f>
@@ -2664,7 +2735,7 @@
         <v>45760525</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="G23" s="22">
         <f>G15+G20</f>
@@ -2693,28 +2764,28 @@
   <sheetData>
     <row r="2" spans="2:4" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" s="15" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="23" t="s">
+        <v>238</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>239</v>
+      </c>
+      <c r="D5" s="23" t="s">
         <v>240</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>241</v>
-      </c>
-      <c r="D5" s="23" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="12" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C6" s="19">
         <v>27291300</v>
@@ -2725,7 +2796,7 @@
     </row>
     <row r="7" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="12" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C7" s="19">
         <v>21542347</v>
@@ -2737,7 +2808,7 @@
     </row>
     <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="12" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C8" s="19">
         <v>5519638</v>
@@ -2749,7 +2820,7 @@
     </row>
     <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="12" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C9" s="19">
         <v>0</v>
@@ -2761,7 +2832,7 @@
     </row>
     <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C10" s="21">
         <f>C6-C7-C8-C9</f>
@@ -2774,7 +2845,7 @@
     </row>
     <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="12" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C11" s="19">
         <v>620800</v>
@@ -2786,7 +2857,7 @@
     </row>
     <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="12" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C12" s="19">
         <v>909616</v>
@@ -2798,7 +2869,7 @@
     </row>
     <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="20" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C13" s="21">
         <f>C10+C11-C12</f>
@@ -2811,7 +2882,7 @@
     </row>
     <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="12" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C14" s="19">
         <v>144542</v>
@@ -2823,7 +2894,7 @@
     </row>
     <row r="15" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="5" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C15" s="22">
         <f>C13-C14</f>
@@ -2836,12 +2907,12 @@
     </row>
     <row r="17" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="18" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="12" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C18" s="19">
         <v>0</v>
@@ -2853,7 +2924,7 @@
     </row>
     <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="20" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C19" s="21">
         <f>C15-C18</f>
@@ -2871,7 +2942,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="B2:D32"/>
+  <dimension ref="B2:D33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -2882,263 +2953,274 @@
   <sheetData>
     <row r="2" spans="2:4" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" s="15" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="23" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="18" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D6" s="15"/>
     </row>
     <row r="7" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="12" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C7" s="27">
         <f>INC_net</f>
         <v>-204043</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="12" t="s">
-        <v>261</v>
-      </c>
-      <c r="C8" s="27">
-        <v>13363219</v>
+        <v>259</v>
+      </c>
+      <c r="C8" s="54">
+        <v>13264120</v>
       </c>
       <c r="D8" s="15" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="C9" s="54">
+        <v>99099</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="28" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="9" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="28" t="s">
-        <v>262</v>
-      </c>
-      <c r="D9" s="15"/>
-    </row>
-    <row r="10" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="12" t="s">
-        <v>263</v>
-      </c>
-      <c r="C10" s="19">
-        <v>-350341</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>264</v>
-      </c>
+      <c r="D10" s="15"/>
     </row>
     <row r="11" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="12" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="C11" s="19">
-        <v>-4858452</v>
+        <v>-350341</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="12" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="12" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C12" s="19">
-        <v>-8199131</v>
+        <v>-4858452</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="12" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C13" s="19">
-        <v>322196</v>
+        <v>-8199131</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C14" s="19">
+        <v>322196</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="C15" s="19">
+        <v>32353</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="20" t="s">
+        <v>267</v>
+      </c>
+      <c r="C16" s="21">
+        <f>SUM(C11:C15)</f>
+        <v>-13053375</v>
+      </c>
+      <c r="D16" s="15"/>
+    </row>
+    <row r="17" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="5" t="s">
         <v>268</v>
       </c>
-      <c r="C14" s="19">
-        <v>32353</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="20" t="s">
+      <c r="C17" s="22">
+        <f>C7+C8+C9+C16</f>
+        <v>105801</v>
+      </c>
+      <c r="D17" s="15"/>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="D18" s="15"/>
+    </row>
+    <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="18" t="s">
         <v>269</v>
-      </c>
-      <c r="C15" s="21">
-        <f>SUM(C10:C14)</f>
-        <v>-13053375</v>
-      </c>
-      <c r="D15" s="15"/>
-    </row>
-    <row r="16" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="5" t="s">
-        <v>270</v>
-      </c>
-      <c r="C16" s="22">
-        <f>C7+C8+C15</f>
-        <v>105801</v>
-      </c>
-      <c r="D16" s="15"/>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="D17" s="15"/>
-    </row>
-    <row r="18" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="18" t="s">
-        <v>271</v>
-      </c>
-      <c r="D18" s="15"/>
-    </row>
-    <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="12" t="s">
-        <v>272</v>
-      </c>
-      <c r="C19" s="19">
-        <v>-124636</v>
       </c>
       <c r="D19" s="15"/>
     </row>
     <row r="20" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="12" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="C20" s="19">
-        <v>721422</v>
+        <v>-124636</v>
       </c>
       <c r="D20" s="15"/>
     </row>
     <row r="21" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="C21" s="19">
+        <v>721422</v>
+      </c>
+      <c r="D21" s="15"/>
+    </row>
+    <row r="22" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="C22" s="19">
+        <v>-924221</v>
+      </c>
+      <c r="D22" s="15"/>
+    </row>
+    <row r="23" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="C23" s="22">
+        <f>SUM(C20:C22)</f>
+        <v>-327435</v>
+      </c>
+      <c r="D23" s="15"/>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="D24" s="15"/>
+    </row>
+    <row r="25" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="18" t="s">
         <v>274</v>
-      </c>
-      <c r="C21" s="19">
-        <v>-924221</v>
-      </c>
-      <c r="D21" s="15"/>
-    </row>
-    <row r="22" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="5" t="s">
-        <v>275</v>
-      </c>
-      <c r="C22" s="22">
-        <f>SUM(C19:C21)</f>
-        <v>-327435</v>
-      </c>
-      <c r="D22" s="15"/>
-    </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="D23" s="15"/>
-    </row>
-    <row r="24" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="18" t="s">
-        <v>276</v>
-      </c>
-      <c r="D24" s="15"/>
-    </row>
-    <row r="25" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="12" t="s">
-        <v>277</v>
-      </c>
-      <c r="C25" s="19">
-        <v>-1294246</v>
       </c>
       <c r="D25" s="15"/>
     </row>
     <row r="26" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="12" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="C26" s="19">
-        <v>2578911</v>
+        <v>-1294246</v>
       </c>
       <c r="D26" s="15"/>
     </row>
     <row r="27" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="12" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="C27" s="19">
-        <v>-19455</v>
+        <v>2578911</v>
       </c>
       <c r="D27" s="15"/>
     </row>
     <row r="28" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="12" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="C28" s="19">
-        <v>347</v>
+        <v>-19455</v>
       </c>
       <c r="D28" s="15"/>
     </row>
     <row r="29" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="C29" s="19">
+        <v>347</v>
+      </c>
+      <c r="D29" s="15"/>
+    </row>
+    <row r="30" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B30" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="C30" s="19">
+        <v>-201123</v>
+      </c>
+      <c r="D30" s="15"/>
+    </row>
+    <row r="31" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B31" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="C31" s="22">
+        <f>SUM(C26:C30)</f>
+        <v>1064434</v>
+      </c>
+      <c r="D31" s="15"/>
+    </row>
+    <row r="32" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B32" s="12" t="s">
+        <v>319</v>
+      </c>
+      <c r="C32" s="45">
+        <v>-55393</v>
+      </c>
+      <c r="D32" s="15"/>
+    </row>
+    <row r="33" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B33" s="5" t="s">
         <v>281</v>
       </c>
-      <c r="C29" s="19">
-        <v>-201123</v>
-      </c>
-      <c r="D29" s="15"/>
-    </row>
-    <row r="30" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B30" s="5" t="s">
-        <v>282</v>
-      </c>
-      <c r="C30" s="22">
-        <f>SUM(C25:C29)</f>
-        <v>1064434</v>
-      </c>
-      <c r="D30" s="15"/>
-    </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B31" s="52" t="s">
-        <v>323</v>
-      </c>
-      <c r="C31" s="53">
-        <v>-55393</v>
-      </c>
-      <c r="D31" s="15"/>
-    </row>
-    <row r="32" spans="2:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B32" s="5" t="s">
-        <v>283</v>
-      </c>
-      <c r="C32" s="22">
-        <f>C16+C22+C30+C31</f>
+      <c r="C33" s="22">
+        <f>C17+C23+C31+C32</f>
         <v>787407</v>
       </c>
-      <c r="D32" s="15"/>
+      <c r="D33" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3158,17 +3240,17 @@
     <col min="6" max="6" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" ht="23" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:6" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B3" s="15" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="23" t="s">
         <v>2</v>
       </c>
@@ -3182,7 +3264,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="12" t="s">
         <v>6</v>
       </c>
@@ -3194,7 +3276,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="12" t="s">
         <v>8</v>
       </c>
@@ -3209,7 +3291,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="12" t="s">
         <v>11</v>
       </c>
@@ -3221,401 +3303,404 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="12" t="s">
-        <v>13</v>
+        <v>340</v>
       </c>
       <c r="C9" s="33">
         <v>962959</v>
       </c>
       <c r="D9" s="30"/>
       <c r="E9" s="30" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="55" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="12" t="s">
         <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="12" t="s">
-        <v>15</v>
       </c>
       <c r="C10" s="34">
         <v>0.09</v>
       </c>
       <c r="D10" s="30"/>
       <c r="E10" s="30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="12" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="12" t="s">
-        <v>17</v>
       </c>
       <c r="C11" s="34">
         <v>0.25</v>
       </c>
       <c r="D11" s="30"/>
       <c r="E11" s="30" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="12" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="12" t="s">
-        <v>19</v>
       </c>
       <c r="C12" s="35">
         <f>share_price*shares_outstanding</f>
         <v>1136291.6199999999</v>
       </c>
       <c r="D12" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="30" t="s">
+    </row>
+    <row r="14" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="52" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="14" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="45" t="s">
+      <c r="C14" s="47"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="47"/>
+    </row>
+    <row r="15" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="12" t="s">
         <v>22</v>
-      </c>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="46"/>
-    </row>
-    <row r="15" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="12" t="s">
-        <v>23</v>
       </c>
       <c r="C15" s="36">
         <f>BAL_equity_shareholders_prior</f>
         <v>13373764</v>
       </c>
       <c r="D15" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="E15" s="30" t="s">
         <v>24</v>
       </c>
-      <c r="E15" s="30" t="s">
+    </row>
+    <row r="16" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="12" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="12" t="s">
-        <v>26</v>
       </c>
       <c r="C16" s="36">
         <f>BAL_inventories_prior</f>
         <v>388718</v>
       </c>
       <c r="D16" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="E16" s="30" t="s">
         <v>27</v>
-      </c>
-      <c r="E16" s="30" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C17" s="36">
         <f>BAL_receivables_prior</f>
         <v>2191178</v>
       </c>
       <c r="D17" s="30" t="s">
+        <v>29</v>
+      </c>
+      <c r="E17" s="30" t="s">
         <v>30</v>
-      </c>
-      <c r="E17" s="30" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C18" s="36">
         <f>BAL_assets_total_prior</f>
         <v>45760525</v>
       </c>
       <c r="D18" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="E18" s="30" t="s">
         <v>33</v>
-      </c>
-      <c r="E18" s="30" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C19" s="36">
         <f>BAL_debt_long_term_prior+BAL_equity_shareholders_prior</f>
         <v>22761169</v>
       </c>
       <c r="D19" s="30" t="s">
+        <v>35</v>
+      </c>
+      <c r="E19" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="E19" s="30" t="s">
+    </row>
+    <row r="21" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="52" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="21" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="45" t="s">
-        <v>38</v>
-      </c>
-      <c r="C21" s="46"/>
-      <c r="D21" s="46"/>
-      <c r="E21" s="46"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="47"/>
+      <c r="E21" s="47"/>
     </row>
     <row r="22" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C22" s="36">
         <f>INC_net+(1-tax_rate)*INC_interest_expense</f>
         <v>478169</v>
       </c>
       <c r="D22" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="E22" s="30" t="s">
         <v>40</v>
-      </c>
-      <c r="E22" s="30" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="23" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C23" s="37">
         <f>IFERROR(INC_sales/365,"")</f>
         <v>74770.684931506854</v>
       </c>
       <c r="D23" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="E23" s="30" t="s">
         <v>43</v>
-      </c>
-      <c r="E23" s="30" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C24" s="36">
         <f>BAL_equity_shareholders_curr</f>
         <v>13308926</v>
       </c>
       <c r="D24" s="30" t="s">
+        <v>45</v>
+      </c>
+      <c r="E24" s="30" t="s">
         <v>46</v>
-      </c>
-      <c r="E24" s="30" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="25" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C25" s="36">
         <f>BAL_cash_marketable_securities_curr</f>
         <v>4354275</v>
       </c>
       <c r="D25" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="E25" s="30" t="s">
         <v>49</v>
-      </c>
-      <c r="E25" s="30" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="26" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C26" s="36">
         <f>BAL_assets_current_curr</f>
         <v>10290295</v>
       </c>
       <c r="D26" s="30" t="s">
+        <v>51</v>
+      </c>
+      <c r="E26" s="30" t="s">
         <v>52</v>
-      </c>
-      <c r="E26" s="30" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="27" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C27" s="36">
         <f>BAL_liabilities_current_curr</f>
         <v>22067307</v>
       </c>
       <c r="D27" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="E27" s="30" t="s">
         <v>55</v>
-      </c>
-      <c r="E27" s="30" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="28" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="12" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C28" s="37">
         <f>IFERROR(INC_cost_goods_sold/365,"")</f>
         <v>59020.128767123286</v>
       </c>
       <c r="D28" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="E28" s="30" t="s">
         <v>58</v>
-      </c>
-      <c r="E28" s="30" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="29" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C29" s="36">
         <f>BAL_debt_long_term_curr</f>
         <v>10080824</v>
       </c>
       <c r="D29" s="30" t="s">
+        <v>60</v>
+      </c>
+      <c r="E29" s="30" t="s">
         <v>61</v>
-      </c>
-      <c r="E29" s="30" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="30" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C30" s="36">
         <f>BAL_assets_current_curr-BAL_liabilities_current_curr</f>
         <v>-11777012</v>
       </c>
       <c r="D30" s="30" t="s">
+        <v>63</v>
+      </c>
+      <c r="E30" s="30" t="s">
         <v>64</v>
-      </c>
-      <c r="E30" s="30" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="31" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C31" s="36">
         <f>BAL_assets_total_curr</f>
         <v>46681735</v>
       </c>
       <c r="D31" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="E31" s="30" t="s">
         <v>67</v>
-      </c>
-      <c r="E31" s="30" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="32" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="12" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C32" s="36">
         <f>BAL_debt_long_term_curr+BAL_equity_shareholders_curr</f>
         <v>23389750</v>
       </c>
       <c r="D32" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="E32" s="30" t="s">
         <v>70</v>
-      </c>
-      <c r="E32" s="30" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="33" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C33" s="36">
         <f>BAL_liabilities_total_curr</f>
         <v>33372809</v>
       </c>
       <c r="D33" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="E33" s="30" t="s">
         <v>73</v>
       </c>
-      <c r="E33" s="30" t="s">
+    </row>
+    <row r="35" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B35" s="52" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="35" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="45" t="s">
-        <v>75</v>
-      </c>
-      <c r="C35" s="46"/>
-      <c r="D35" s="46"/>
-      <c r="E35" s="46"/>
+      <c r="C35" s="47"/>
+      <c r="D35" s="47"/>
+      <c r="E35" s="47"/>
     </row>
     <row r="36" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B36" s="12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C36" s="37">
         <f>AVERAGE(startYear_equity,currentYear_equity)</f>
         <v>13341345</v>
       </c>
       <c r="D36" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="E36" s="30" t="s">
         <v>77</v>
-      </c>
-      <c r="E36" s="30" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="37" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C37" s="37">
         <f>AVERAGE(startYear_total_assets,currentYear_assets_total)</f>
         <v>46221130</v>
       </c>
       <c r="D37" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="E37" s="30" t="s">
         <v>80</v>
-      </c>
-      <c r="E37" s="30" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="38" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C38" s="37">
         <f>AVERAGE(startYear_total_capitalization,currentYear_total_capitalization)</f>
         <v>23075459.5</v>
       </c>
       <c r="D38" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="E38" s="30" t="s">
         <v>83</v>
-      </c>
-      <c r="E38" s="30" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="41" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B41" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="C41" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="C41" s="23" t="s">
+      <c r="D41" s="23" t="s">
         <v>86</v>
-      </c>
-      <c r="D41" s="23" t="s">
-        <v>87</v>
       </c>
       <c r="E41" s="23" t="s">
         <v>5</v>
       </c>
       <c r="F41" s="23" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="42" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B42" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
@@ -3623,46 +3708,46 @@
     </row>
     <row r="43" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B43" s="12" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C43" s="38">
         <f>market_capitalization - currentYear_equity</f>
         <v>-12172634.380000001</v>
       </c>
       <c r="D43" s="30" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E43" s="30"/>
     </row>
     <row r="44" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B44" s="12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C44" s="39">
         <f>market_capitalization / currentYear_equity</f>
         <v>8.5378160491688046E-2</v>
       </c>
       <c r="D44" s="30" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E44" s="30"/>
     </row>
     <row r="45" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B45" s="12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C45" s="38">
         <f>currentYear_after_tax_operating_income-(cost_capital*startYear_total_capitalization)</f>
         <v>-1570336.21</v>
       </c>
       <c r="D45" s="30" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E45" s="30"/>
     </row>
     <row r="46" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B46" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C46" s="1"/>
       <c r="D46" s="1"/>
@@ -3670,85 +3755,85 @@
     </row>
     <row r="47" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B47" s="12" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C47" s="40">
         <f>currentYear_after_tax_operating_income/startYear_total_assets</f>
         <v>1.0449377492937418E-2</v>
       </c>
       <c r="D47" s="30" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E47" s="30"/>
     </row>
     <row r="48" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B48" s="12" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C48" s="40">
         <f>currentYear_after_tax_operating_income/startYear_total_capitalization</f>
         <v>2.1008103757763935E-2</v>
       </c>
       <c r="D48" s="30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E48" s="30"/>
     </row>
     <row r="49" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B49" s="12" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C49" s="40">
         <f>INC_net/startYear_equity</f>
         <v>-1.5256961316200884E-2</v>
       </c>
       <c r="D49" s="30" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E49" s="30"/>
     </row>
     <row r="50" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B50" s="12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C50" s="40">
         <f>currentYear_after_tax_operating_income/avg_total_assets</f>
         <v>1.0345246860039986E-2</v>
       </c>
       <c r="D50" s="30" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E50" s="30"/>
     </row>
     <row r="51" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B51" s="12" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C51" s="40">
         <f>currentYear_after_tax_operating_income/avg_total_capitalization</f>
         <v>2.0721970888597039E-2</v>
       </c>
       <c r="D51" s="30" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E51" s="30"/>
     </row>
     <row r="52" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B52" s="12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C52" s="40">
         <f>INC_net/avg_equity</f>
         <v>-1.5294035196601241E-2</v>
       </c>
       <c r="D52" s="30" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E52" s="30"/>
     </row>
     <row r="53" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B53" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C53" s="1"/>
       <c r="D53" s="1"/>
@@ -3756,102 +3841,102 @@
     </row>
     <row r="54" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B54" s="12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C54" s="39">
         <f>INC_sales/startYear_total_assets</f>
         <v>0.59639394434395143</v>
       </c>
       <c r="D54" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="E54" s="30" t="s">
         <v>111</v>
-      </c>
-      <c r="E54" s="30" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="55" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B55" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C55" s="39">
         <f>INC_sales/startYear_receivables</f>
         <v>12.455081239406383</v>
       </c>
       <c r="D55" s="30" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E55" s="30"/>
     </row>
     <row r="56" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B56" s="12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C56" s="41">
         <f>startYear_receivables/currentYear_daily_sales_average</f>
         <v>29.305308651475009</v>
       </c>
       <c r="D56" s="30" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E56" s="30"/>
     </row>
     <row r="57" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B57" s="12" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C57" s="39">
         <f>INC_cost_goods_sold/startYear_inventory</f>
         <v>55.418959245519886</v>
       </c>
       <c r="D57" s="30" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E57" s="30"/>
     </row>
     <row r="58" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B58" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C58" s="41">
         <f>startYear_inventory/currentYear_cost_goods_sold_daily</f>
         <v>6.5861936956080047</v>
       </c>
       <c r="D58" s="30" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E58" s="30"/>
     </row>
     <row r="59" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59" s="12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C59" s="40">
         <f>INC_net/INC_sales</f>
         <v>-7.47648518025891E-3</v>
       </c>
       <c r="D59" s="30" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E59" s="30"/>
     </row>
     <row r="60" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B60" s="12" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C60" s="40">
         <f>currentYear_after_tax_operating_income/INC_sales</f>
         <v>1.7520931578928083E-2</v>
       </c>
       <c r="D60" s="30" t="s">
+        <v>123</v>
+      </c>
+      <c r="E60" s="30" t="s">
         <v>124</v>
-      </c>
-      <c r="E60" s="30" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="61" spans="2:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B61" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
@@ -3859,102 +3944,104 @@
     </row>
     <row r="62" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B62" s="12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C62" s="40">
         <f>currentYear_debt_long_term/(currentYear_debt_long_term+currentYear_equity)</f>
         <v>0.4309932342158424</v>
       </c>
       <c r="D62" s="30" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E62" s="30"/>
     </row>
     <row r="63" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B63" s="12" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C63" s="39">
         <f>currentYear_debt_long_term/currentYear_equity</f>
         <v>0.75744834707173214</v>
       </c>
       <c r="D63" s="30" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E63" s="30"/>
     </row>
     <row r="64" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B64" s="12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C64" s="40">
         <f>currentYear_liabilities_total/currentYear_assets_total</f>
         <v>0.71490078507150601</v>
       </c>
       <c r="D64" s="30" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E64" s="30"/>
     </row>
     <row r="65" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B65" s="12" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C65" s="39">
         <f>INC_ebit/INC_interest_expense</f>
         <v>0.25210088652794144</v>
       </c>
       <c r="D65" s="30" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E65" s="30"/>
     </row>
     <row r="66" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B66" s="12" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C66" s="39">
-        <f>(INC_ebit+INC_depreciation)/INC_interest_expense</f>
-        <v>0.25210088652794144</v>
+        <f>(INC_ebit+CF_depreciation_amortization)/INC_interest_expense</f>
+        <v>14.834210260153736</v>
       </c>
       <c r="D66" s="30" t="s">
-        <v>136</v>
-      </c>
-      <c r="E66" s="30"/>
+        <v>342</v>
+      </c>
+      <c r="E66" s="30" t="s">
+        <v>343</v>
+      </c>
     </row>
     <row r="67" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B67" s="12" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C67" s="42">
         <f>INC_net/currentYear_after_tax_operating_income</f>
         <v>-0.42671733215662244</v>
       </c>
       <c r="D67" s="30" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E67" s="30" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="68" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B68" s="12" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C68" s="39">
         <f>currentYear_assets_total/currentYear_equity</f>
         <v>3.5075508722491957</v>
       </c>
       <c r="D68" s="30" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E68" s="30" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="69" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B69" s="5" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C69" s="1"/>
       <c r="D69" s="1"/>
@@ -3962,59 +4049,59 @@
     </row>
     <row r="70" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B70" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C70" s="40">
         <f>currentYear_working_capital_net/currentYear_assets_total</f>
         <v>-0.25228308245184117</v>
       </c>
       <c r="D70" s="30" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E70" s="30"/>
     </row>
     <row r="71" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B71" s="12" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C71" s="39">
         <f>currentYear_assets_current/currentYear_liabilities_current</f>
         <v>0.46631403641595232</v>
       </c>
       <c r="D71" s="30" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E71" s="30"/>
     </row>
     <row r="72" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B72" s="12" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C72" s="39">
         <f>(currentYear_cash_marketable_securities+BAL_receivables_curr)/currentYear_liabilities_current</f>
         <v>0.31163489953712975</v>
       </c>
       <c r="D72" s="30" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E72" s="30"/>
     </row>
     <row r="73" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B73" s="12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C73" s="39">
         <f>currentYear_cash_marketable_securities/currentYear_liabilities_current</f>
         <v>0.19731791468709797</v>
       </c>
       <c r="D73" s="30" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E73" s="30"/>
     </row>
     <row r="74" spans="2:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B74" s="5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C74" s="1"/>
       <c r="D74" s="1"/>
@@ -4022,14 +4109,14 @@
     </row>
     <row r="75" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B75" s="12" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C75" s="40">
         <f>RATIO_asset_turnover*RATIO_operating_profit_margin</f>
         <v>1.0449377492937416E-2</v>
       </c>
       <c r="D75" s="30" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E75" s="30"/>
       <c r="F75" s="44" t="str">
@@ -4039,14 +4126,14 @@
     </row>
     <row r="76" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B76" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C76" s="40">
         <f>RATIO_leverage*RATIO_asset_turnover*RATIO_operating_profit_margin*RATIO_debt_burden</f>
         <v>-1.5639925517164466E-2</v>
       </c>
       <c r="D76" s="30" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E76" s="30"/>
     </row>
@@ -4062,7 +4149,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="B2:D24"/>
+  <dimension ref="B2:D26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.83203125" customWidth="1"/>
@@ -4073,206 +4160,228 @@
   <sheetData>
     <row r="2" spans="2:4" ht="23" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="14" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C2" s="14"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B4" s="43" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C4" s="43" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B5" s="43" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C5" s="43" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B6" s="43" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C6" s="43" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B7" s="43" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C7" s="43" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B8" s="43" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C8" s="43" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.2">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" ht="75" x14ac:dyDescent="0.2">
       <c r="B9" s="43" t="s">
-        <v>294</v>
-      </c>
-      <c r="C9" s="43" t="s">
-        <v>329</v>
+        <v>344</v>
+      </c>
+      <c r="C9" s="53" t="s">
+        <v>345</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.2">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" ht="30" x14ac:dyDescent="0.2">
       <c r="B10" s="43" t="s">
-        <v>296</v>
+        <v>347</v>
       </c>
       <c r="C10" s="43" t="s">
-        <v>330</v>
+        <v>348</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>209</v>
+        <v>349</v>
       </c>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B11" s="43" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="C11" s="43" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>298</v>
+        <v>207</v>
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B12" s="43" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="C12" s="43" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B13" s="43" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="C13" s="43" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B14" s="43" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="C14" s="43" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B16" s="43" t="s">
-        <v>305</v>
-      </c>
-      <c r="C16" s="43"/>
-      <c r="D16" s="4" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B15" s="43" t="s">
+        <v>299</v>
+      </c>
+      <c r="C15" s="43" t="s">
+        <v>329</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B17" s="43" t="s">
-        <v>307</v>
-      </c>
-      <c r="C17" s="43" t="s">
-        <v>335</v>
-      </c>
+        <v>301</v>
+      </c>
+      <c r="C17" s="43"/>
       <c r="D17" s="4" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="43" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="C18" s="43" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="43" t="s">
-        <v>311</v>
-      </c>
-      <c r="C19" s="43" t="s">
-        <v>336</v>
+        <v>305</v>
+      </c>
+      <c r="C19" s="53" t="s">
+        <v>332</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="29" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="43" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="C20" s="43" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B22" s="43" t="s">
-        <v>315</v>
-      </c>
-      <c r="C22" s="43"/>
-    </row>
-    <row r="23" spans="2:4" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="43" t="s">
+        <v>309</v>
+      </c>
+      <c r="C21" s="43" t="s">
+        <v>331</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B23" s="43" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="C23" s="43"/>
-      <c r="D23" s="4" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="24" spans="2:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="2:4" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="43" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="C24" s="43"/>
       <c r="D24" s="4" t="s">
-        <v>319</v>
+        <v>313</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="43" t="s">
+        <v>314</v>
+      </c>
+      <c r="C25" s="43"/>
+      <c r="D25" s="4" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="43" t="s">
+        <v>335</v>
+      </c>
+      <c r="C26" s="43" t="s">
+        <v>336</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>